<commit_message>
data: update records 2026-08-17
</commit_message>
<xml_diff>
--- a/public/records.xlsx
+++ b/public/records.xlsx
@@ -863,27 +863,27 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>54.07</t>
+          <t>54.06</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>54.07</t>
+          <t>54.06</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Мюнхен</t>
+          <t>Париж</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>10.07.2026</t>
+          <t>12.08.2026</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -1055,27 +1055,27 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>1:58.06</t>
+          <t>1:57.10</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>118.06</t>
+          <t>117.10</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Санкт-Петербург</t>
+          <t>Париж</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>19.04.2026</t>
+          <t>10.08.2026</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
@@ -3199,27 +3199,27 @@
       <c r="E57" t="inlineStr"/>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>1:57.07</t>
+          <t>1:56.16</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>117.07</t>
+          <t>116.16</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Мюнхен</t>
+          <t>Париж</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>08.07.2026</t>
+          <t>16.08.2026</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
@@ -5167,17 +5167,17 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>54.07</t>
+          <t>54.06</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Мюнхен</t>
+          <t>Париж</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10.07.2026</t>
+          <t>12.08.2026</t>
         </is>
       </c>
     </row>
@@ -5279,17 +5279,17 @@
       <c r="C13" t="inlineStr"/>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>1:58.06</t>
+          <t>1:57.10</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Санкт-Петербург</t>
+          <t>Париж</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>19.04.2026</t>
+          <t>10.08.2026</t>
         </is>
       </c>
     </row>
@@ -6651,17 +6651,17 @@
       <c r="C14" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>1:57.07</t>
+          <t>1:56.16</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Мюнхен</t>
+          <t>Париж</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08.07.2026</t>
+          <t>16.08.2026</t>
         </is>
       </c>
     </row>

</xml_diff>